<commit_message>
Update アクションプランシート.xlsx with full training content
研修全内容（受容・認める技術・心理的安全性・成功循環モデル等）を反映した記入済みシートに更新。

https://claude.ai/code/session_01B9dtUvo4j9tUD9LrREQnFg
</commit_message>
<xml_diff>
--- a/アクションプランシート.xlsx
+++ b/アクションプランシート.xlsx
@@ -44,8 +44,8 @@
     </font>
     <font>
       <name val="Meiryo"/>
-      <color rgb="00222222"/>
-      <sz val="10"/>
+      <color rgb="001a1a1a"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Meiryo"/>
@@ -495,22 +495,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A2:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
     <col width="2" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="1" ht="8" customHeight="1"/>
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -530,34 +525,88 @@
       <c r="C3" s="1" t="n"/>
       <c r="D3" s="1" t="n"/>
     </row>
-    <row r="4" ht="80" customHeight="1">
+    <row r="4" ht="115" customHeight="1">
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>研修を通じて、気づいたこと、学んだこと</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>【受容と返報性の法則】
+・カール・ロジャーズの言葉「正そうとする前に、わかろうとせよ」が強く印象に残った。
+　部下を変えようとする前に、まず相手の立場・想いを理解する姿勢が信頼関係の土台になる。
+・「受け入れてから受け入れられる」—— 自分がまず相手を受け容れることで、返報性の法則が働き、
+　相手も自分を受け入れてくれるようになることを学んだ。
+【認める技術 ４段階】
+　①存在承認（存在そのものを認める） ②事実承認（努力・プロセスを認める）
+　③変化承認（良い方向の変化を認める） ④成果承認（結果を認める）
+　⇒ これまで④成果承認に偏りがちで、①②③が不足していたと気づいた。
+【心理的安全性とチームの生産性】
+・Googleのプロジェクト・アリストテレス：個人の能力よりチームの『心理的安全性』が
+　生産性向上の最重要因子であることを学んだ。
+・心理的安全性が低いと「無知・無能・邪魔・ネガティブと思われる不安」が生じ、
+　発言・報告・提案ができなくなる。
+【組織の成功循環モデル（ダニエル・キム）】
+・「関係の質」→「思考の質」→「行動の質」→「結果の質」の良い循環が重要。
+　結果ばかりを求めると悪い循環に陥る。まず「関係の質」を高めることが出発点。
+・「何もしていない」はネガティブ。コミュニケーションで最もしてはいけないことは『無視』。</t>
+        </is>
+      </c>
       <c r="D4" s="1" t="n"/>
     </row>
-    <row r="5" ht="80" customHeight="1">
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="6" t="inlineStr">
         <is>
           <t>自分自身が実践しようと思うこと</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>【アクティブ・リスニングの実践】
+・部下・メンバーと話す際、うなずき・オウム返し・「それで？」を意識して、
+　相手が話し終わるまで最後まで聴く。
+【認める言動を増やす】
+・毎日1回、意識してメンバーへ声をかける（存在承認）。
+・「ありがとう」「助かった」「さすがだね」「君なら出来る」などポジティブな言葉を積極的に使う。
+・結果だけでなく、努力・プロセス・変化を具体的な言葉で伝える（事実承認・変化承認）。
+　例：「先週より〇〇がスムーズになったね」「毎回丁寧に準備してくれているね」
+【受容の姿勢】
+・指摘・修正の前に「まず相手を理解しようとする」を徹底する。
+　（正す前に、わかろうとせよ）
+【関係の質を意識した日常行動】
+・笑顔で挨拶する、目を見て話を聴く、メモしながら聴くなど非言語のポジティブ行動を習慣化する。</t>
+        </is>
+      </c>
       <c r="D5" s="1" t="n"/>
     </row>
-    <row r="6" ht="80" customHeight="1">
+    <row r="6" ht="100" customHeight="1">
       <c r="A6" s="1" t="n"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
           <t>会社全体や部署、チームの皆と実践しようと思うこと</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>【心理的安全性の高い職場づくり】
+・誰もが発言・相談しやすい雰囲気をチーム全体でつくる。
+・ミスや失敗を責める文化をなくし、「報告・相談しやすい環境」を整える。
+【認め合う文化の醸成】
+・ミーティングの冒頭で「メンバーの良い行動・変化」を称え合う時間を設ける。
+・「感謝の気持ちを伝える」文化を部署全体に広げる。
+【良い循環をつくる仕組み化】
+・定期的な1on1ミーティングを導入し、メンバー一人ひとりの想いや課題を
+　受容・傾聴する場をつくる。
+・上位者・先輩が後輩・部下に寄り添い、サポートし合う文化をつくる。
+　（帝京大学ラグビー・広島カープの事例：助け合い・リスペクト・連帯感）
+【チームとして目標を共有する】
+・チームの目標と各自の役割を全員で共有し、「このチームのために何かしたい」
+　という当事者意識が生まれる環境をつくる。</t>
+        </is>
+      </c>
       <c r="D6" s="1" t="n"/>
     </row>
     <row r="7" ht="14" customHeight="1">
@@ -574,12 +623,7 @@
       </c>
       <c r="D7" s="1" t="n"/>
     </row>
-    <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
-    </row>
+    <row r="8" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B3:C3"/>

</xml_diff>

<commit_message>
Update アクションプランシート.xlsx with gas station-specific content
ガソリンスタンドの業務（給油・接客・スタッフ管理・ヒヤリハット等）に落とし込んだ内容に更新。

https://claude.ai/code/session_01B9dtUvo4j9tUD9LrREQnFg
</commit_message>
<xml_diff>
--- a/アクションプランシート.xlsx
+++ b/アクションプランシート.xlsx
@@ -525,7 +525,7 @@
       <c r="C3" s="1" t="n"/>
       <c r="D3" s="1" t="n"/>
     </row>
-    <row r="4" ht="115" customHeight="1">
+    <row r="4" ht="118" customHeight="1">
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="6" t="inlineStr">
         <is>
@@ -534,29 +534,27 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>【受容と返報性の法則】
-・カール・ロジャーズの言葉「正そうとする前に、わかろうとせよ」が強く印象に残った。
-　部下を変えようとする前に、まず相手の立場・想いを理解する姿勢が信頼関係の土台になる。
-・「受け入れてから受け入れられる」—— 自分がまず相手を受け容れることで、返報性の法則が働き、
-　相手も自分を受け入れてくれるようになることを学んだ。
-【認める技術 ４段階】
-　①存在承認（存在そのものを認める） ②事実承認（努力・プロセスを認める）
-　③変化承認（良い方向の変化を認める） ④成果承認（結果を認める）
-　⇒ これまで④成果承認に偏りがちで、①②③が不足していたと気づいた。
-【心理的安全性とチームの生産性】
-・Googleのプロジェクト・アリストテレス：個人の能力よりチームの『心理的安全性』が
-　生産性向上の最重要因子であることを学んだ。
-・心理的安全性が低いと「無知・無能・邪魔・ネガティブと思われる不安」が生じ、
-　発言・報告・提案ができなくなる。
-【組織の成功循環モデル（ダニエル・キム）】
-・「関係の質」→「思考の質」→「行動の質」→「結果の質」の良い循環が重要。
-　結果ばかりを求めると悪い循環に陥る。まず「関係の質」を高めることが出発点。
-・「何もしていない」はネガティブ。コミュニケーションで最もしてはいけないことは『無視』。</t>
+          <t>【お客様対応への気づき】
+・給油案内・洗車提案・オイル交換の声かけなど、日々の接客が「存在承認」の積み重ねだと気づいた。
+　お客様の名前を覚えて挨拶するだけでも「自分のことを見てくれている」という信頼感につながる。
+・「返報性の法則」を実感：こちらから笑顔・挨拶・感謝を先に示すことで、
+　リピーターやサービス購入につながることを改めて認識した。
+【スタッフマネジメントへの気づき】
+・給油ミス・釣り銭ミス・ヒヤリハットを「報告しにくい雰囲気」が続くと、大きな事故につながる。
+　心理的安全性の低い職場では「無能と思われる不安」「怒られる不安」でミス隠しが起きると気づいた。
+・スタッフへの承認が「成果承認（販売件数・洗車台数）」に偏っていた。
+　新人が丁寧に窓拭きをした、接客言葉が改善されたなど
+　「事実承認・変化承認」をもっと伝えるべきだったと気づいた。
+【チーム・組織への気づき】
+・結果（売上・台数）を先に求めると、スタッフが萎縮して自発性がなくなる（悪い循環）。
+　まずスタッフ同士の「関係の質」を高めることが、自然と接客品質・業績向上につながる（良い循環）。
+・「何もしていない（無視）」が最もチームの雰囲気を悪化させる。
+　シフトの中でも声かけ・感謝を意識することが管理職の重要な役割だと学んだ。</t>
         </is>
       </c>
       <c r="D4" s="1" t="n"/>
     </row>
-    <row r="5" ht="100" customHeight="1">
+    <row r="5" ht="105" customHeight="1">
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="6" t="inlineStr">
         <is>
@@ -565,24 +563,26 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>【アクティブ・リスニングの実践】
-・部下・メンバーと話す際、うなずき・オウム返し・「それで？」を意識して、
-　相手が話し終わるまで最後まで聴く。
-【認める言動を増やす】
-・毎日1回、意識してメンバーへ声をかける（存在承認）。
-・「ありがとう」「助かった」「さすがだね」「君なら出来る」などポジティブな言葉を積極的に使う。
-・結果だけでなく、努力・プロセス・変化を具体的な言葉で伝える（事実承認・変化承認）。
-　例：「先週より〇〇がスムーズになったね」「毎回丁寧に準備してくれているね」
-【受容の姿勢】
-・指摘・修正の前に「まず相手を理解しようとする」を徹底する。
-　（正す前に、わかろうとせよ）
-【関係の質を意識した日常行動】
-・笑顔で挨拶する、目を見て話を聴く、メモしながら聴くなど非言語のポジティブ行動を習慣化する。</t>
+          <t>【スタッフへの声かけ・承認】
+・出勤時・シフト開始時に必ず全スタッフへ一言声をかける（存在承認の習慣化）。
+・接客態度が改善されたスタッフ、丁寧な作業をしたスタッフに
+　「さっきの対応よかったよ」と具体的に伝える（事実承認・変化承認）。
+【ミス・相談への対応を変える】
+・給油ミスやクレームが起きたとき、まず「何があったか聞く」を徹底する。
+　（叱る前に、まずわかろうとせよ ＝ カール・ロジャーズの教え）
+・新人スタッフが質問しやすいよう、「聞いてくれてよかった」と返す言葉を意識する。
+【接客でのアクティブ・リスニング実践】
+・お客様からのご要望・ご不満を聴く際、うなずき・オウム返しで
+　「きちんと聴いている」姿勢を示す。
+　例：「タイヤの空気が減ってきた気がして…」→「タイヤの空気が気になっていらっしゃるんですね」
+【ポジティブ言語を増やす】
+・「ありがとう」「助かった」「さすが」を1日の中で意識して使う。
+　「なんでできないんだ」「またミスか」などネガティブな言葉を使わないよう気をつける。</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
     </row>
-    <row r="6" ht="100" customHeight="1">
+    <row r="6" ht="105" customHeight="1">
       <c r="A6" s="1" t="n"/>
       <c r="B6" s="6" t="inlineStr">
         <is>
@@ -591,20 +591,21 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>【心理的安全性の高い職場づくり】
-・誰もが発言・相談しやすい雰囲気をチーム全体でつくる。
-・ミスや失敗を責める文化をなくし、「報告・相談しやすい環境」を整える。
-【認め合う文化の醸成】
-・ミーティングの冒頭で「メンバーの良い行動・変化」を称え合う時間を設ける。
-・「感謝の気持ちを伝える」文化を部署全体に広げる。
-【良い循環をつくる仕組み化】
-・定期的な1on1ミーティングを導入し、メンバー一人ひとりの想いや課題を
-　受容・傾聴する場をつくる。
-・上位者・先輩が後輩・部下に寄り添い、サポートし合う文化をつくる。
-　（帝京大学ラグビー・広島カープの事例：助け合い・リスペクト・連帯感）
-【チームとして目標を共有する】
-・チームの目標と各自の役割を全員で共有し、「このチームのために何かしたい」
-　という当事者意識が生まれる環境をつくる。</t>
+          <t>【心理的安全性の高いスタンドづくり】
+・ヒヤリハット・小さなミスを「報告してよかった」と思える雰囲気をチーム全体でつくる。
+　（報告・連絡・相談がしやすい職場 ＝ 安全な職場・良いサービスの土台）
+【認め合う文化の導入】
+・朝礼・夕礼の中で「今日よかったこと・頑張ったスタッフ」を一言称え合う時間を設ける。
+・申し送りノートに「良かった接客・工夫した点」を記録する欄を追加し、
+　スタッフ同士がお互いを認め合う習慣をつくる。
+【先輩が後輩をサポートする文化】
+・経験あるスタッフが新人・若手に寄り添い「伴走」する姿勢を全体で共有する。
+　（帝京大学ラグビー・広島カープの事例：助け合い・リスペクトが常勝チームをつくる）
+【チーム目標の共有】
+・洗車台数・油外収益などの目標を全スタッフで共有し、
+　「自分もこのチームの力になりたい」という当事者意識が生まれる場をつくる。
+・結果だけを追求するのではなく、「関係の質→思考の質→行動の質→結果」の
+　良い循環をスタンド全体で意識していく。</t>
         </is>
       </c>
       <c r="D6" s="1" t="n"/>

</xml_diff>